<commit_message>
Hoàn thiện thay nút ISO
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/02-FRM-200/FRM-201_RFQ_Register.xlsx
+++ b/04-Bieu-Mau/02-FRM-200/FRM-201_RFQ_Register.xlsx
@@ -4,11 +4,11 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM-201_LOG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_LISTS" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_IMPORT" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILTER_VIEW" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_LISTS" sheetId="2" state="veryHidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_IMPORT" sheetId="3" state="veryHidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILTER_VIEW" sheetId="4" state="veryHidden" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERIOD_REVIEW" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REF_LINKS" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REF_LINKS" sheetId="6" state="veryHidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="VAL_STATUS_CORE">'_LISTS'!$A$2:$A$7</definedName>
@@ -4560,7 +4560,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="80" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="693">
+  <cellXfs count="700">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -6274,6 +6274,25 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="335" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="139" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="120" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="121" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="57" fillId="4" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -6372,6 +6391,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6402,6 +6424,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6432,6 +6457,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -6764,18 +6792,18 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="340" t="n"/>
-      <c r="B1" s="53" t="n"/>
+      <c r="A1" s="412" t="n"/>
+      <c r="B1" s="310" t="n"/>
       <c r="C1" s="3" t="inlineStr">
         <is>
           <t>RFQ REGISTER</t>
         </is>
       </c>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="D1" s="268" t="n"/>
+      <c r="E1" s="268" t="n"/>
+      <c r="F1" s="268" t="n"/>
+      <c r="G1" s="268" t="n"/>
+      <c r="H1" s="268" t="n"/>
       <c r="I1" s="621" t="inlineStr">
         <is>
           <t>Form Code</t>
@@ -6818,14 +6846,9 @@
       <c r="AN1" s="625" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="9" t="n"/>
-      <c r="B2" s="54" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="10" t="n"/>
-      <c r="H2" s="10" t="n"/>
+      <c r="A2" s="275" t="n"/>
+      <c r="B2" s="312" t="n"/>
+      <c r="C2" s="275" t="n"/>
       <c r="I2" s="626" t="inlineStr">
         <is>
           <t>Revision</t>
@@ -6868,14 +6891,9 @@
       <c r="AN2" s="630" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="54" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
+      <c r="A3" s="275" t="n"/>
+      <c r="B3" s="312" t="n"/>
+      <c r="C3" s="275" t="n"/>
       <c r="I3" s="626" t="inlineStr">
         <is>
           <t>Eff. Date</t>
@@ -6918,18 +6936,13 @@
       <c r="AN3" s="630" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="9" t="n"/>
-      <c r="B4" s="54" t="n"/>
+      <c r="A4" s="275" t="n"/>
+      <c r="B4" s="312" t="n"/>
       <c r="C4" s="631" t="inlineStr">
         <is>
           <t>Quality Management System  ·  Controlled Document</t>
         </is>
       </c>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
       <c r="I4" s="632" t="inlineStr">
         <is>
           <t>Owner</t>
@@ -6972,18 +6985,18 @@
       <c r="AN4" s="630" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="18" t="n"/>
-      <c r="B5" s="24" t="n"/>
+      <c r="A5" s="282" t="n"/>
+      <c r="B5" s="287" t="n"/>
       <c r="C5" s="634" t="inlineStr">
         <is>
           <t>HESEM Engineering  ·  ISO 9001 / AS9100  ·  Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="19" t="n"/>
-      <c r="F5" s="19" t="n"/>
-      <c r="G5" s="19" t="n"/>
-      <c r="H5" s="19" t="n"/>
+      <c r="D5" s="283" t="n"/>
+      <c r="E5" s="283" t="n"/>
+      <c r="F5" s="283" t="n"/>
+      <c r="G5" s="283" t="n"/>
+      <c r="H5" s="283" t="n"/>
       <c r="I5" s="635" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -7073,15 +7086,15 @@
           <t>1.  RFQ INTAKE BLOCK</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n"/>
-      <c r="C7" s="27" t="n"/>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
-      <c r="H7" s="27" t="n"/>
-      <c r="I7" s="27" t="n"/>
-      <c r="J7" s="27" t="n"/>
+      <c r="B7" s="289" t="n"/>
+      <c r="C7" s="289" t="n"/>
+      <c r="D7" s="289" t="n"/>
+      <c r="E7" s="289" t="n"/>
+      <c r="F7" s="289" t="n"/>
+      <c r="G7" s="289" t="n"/>
+      <c r="H7" s="289" t="n"/>
+      <c r="I7" s="289" t="n"/>
+      <c r="J7" s="289" t="n"/>
       <c r="K7" s="643" t="n"/>
       <c r="L7" s="643" t="n"/>
       <c r="M7" s="643" t="n"/>
@@ -7114,24 +7127,24 @@
       <c r="AN7" s="644" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="645" t="inlineStr">
+      <c r="A8" s="685" t="inlineStr">
         <is>
           <t>Open Period</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="646" t="inlineStr"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="647" t="inlineStr">
+      <c r="B8" s="272" t="n"/>
+      <c r="C8" s="331" t="inlineStr"/>
+      <c r="D8" s="271" t="n"/>
+      <c r="E8" s="272" t="n"/>
+      <c r="F8" s="686" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="646" t="inlineStr"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="6" t="n"/>
+      <c r="G8" s="272" t="n"/>
+      <c r="H8" s="331" t="inlineStr"/>
+      <c r="I8" s="271" t="n"/>
+      <c r="J8" s="272" t="n"/>
       <c r="K8" s="648" t="n"/>
       <c r="L8" s="648" t="n"/>
       <c r="M8" s="648" t="n"/>
@@ -7164,24 +7177,24 @@
       <c r="AN8" s="649" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="650" t="inlineStr">
+      <c r="A9" s="687" t="inlineStr">
         <is>
           <t>Commercial Owner</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="651" t="inlineStr"/>
-      <c r="D9" s="12" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="652" t="inlineStr">
+      <c r="B9" s="278" t="n"/>
+      <c r="C9" s="693" t="inlineStr"/>
+      <c r="D9" s="277" t="n"/>
+      <c r="E9" s="278" t="n"/>
+      <c r="F9" s="688" t="inlineStr">
         <is>
           <t>Part No. / Revision</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n"/>
-      <c r="H9" s="651" t="inlineStr"/>
-      <c r="I9" s="12" t="n"/>
-      <c r="J9" s="13" t="n"/>
+      <c r="G9" s="278" t="n"/>
+      <c r="H9" s="693" t="inlineStr"/>
+      <c r="I9" s="277" t="n"/>
+      <c r="J9" s="278" t="n"/>
       <c r="K9" s="653" t="n"/>
       <c r="L9" s="653" t="n"/>
       <c r="M9" s="653" t="n"/>
@@ -7214,24 +7227,24 @@
       <c r="AN9" s="654" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="650" t="inlineStr">
+      <c r="A10" s="687" t="inlineStr">
         <is>
           <t>Evidence Folder</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="651" t="inlineStr"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="652" t="inlineStr">
+      <c r="B10" s="278" t="n"/>
+      <c r="C10" s="693" t="inlineStr"/>
+      <c r="D10" s="277" t="n"/>
+      <c r="E10" s="278" t="n"/>
+      <c r="F10" s="688" t="inlineStr">
         <is>
           <t>RFQ Outcome</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n"/>
-      <c r="H10" s="651" t="inlineStr"/>
-      <c r="I10" s="12" t="n"/>
-      <c r="J10" s="13" t="n"/>
+      <c r="G10" s="278" t="n"/>
+      <c r="H10" s="693" t="inlineStr"/>
+      <c r="I10" s="277" t="n"/>
+      <c r="J10" s="278" t="n"/>
       <c r="K10" s="653" t="n"/>
       <c r="L10" s="653" t="n"/>
       <c r="M10" s="653" t="n"/>
@@ -7264,24 +7277,24 @@
       <c r="AN10" s="654" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="650" t="inlineStr">
+      <c r="A11" s="687" t="inlineStr">
         <is>
           <t>Next Review Date</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="651" t="inlineStr"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="652" t="inlineStr">
+      <c r="B11" s="278" t="n"/>
+      <c r="C11" s="693" t="inlineStr"/>
+      <c r="D11" s="277" t="n"/>
+      <c r="E11" s="278" t="n"/>
+      <c r="F11" s="688" t="inlineStr">
         <is>
           <t>Risk Level</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n"/>
-      <c r="H11" s="651" t="inlineStr"/>
-      <c r="I11" s="12" t="n"/>
-      <c r="J11" s="13" t="n"/>
+      <c r="G11" s="278" t="n"/>
+      <c r="H11" s="693" t="inlineStr"/>
+      <c r="I11" s="277" t="n"/>
+      <c r="J11" s="278" t="n"/>
       <c r="K11" s="655" t="n"/>
       <c r="L11" s="655" t="n"/>
       <c r="M11" s="655" t="n"/>
@@ -7314,24 +7327,24 @@
       <c r="AN11" s="656" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="657" t="inlineStr">
+      <c r="A12" s="689" t="inlineStr">
         <is>
           <t>Process Owner</t>
         </is>
       </c>
-      <c r="B12" s="22" t="n"/>
-      <c r="C12" s="658" t="inlineStr"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="22" t="n"/>
-      <c r="F12" s="659" t="inlineStr">
+      <c r="B12" s="285" t="n"/>
+      <c r="C12" s="694" t="inlineStr"/>
+      <c r="D12" s="283" t="n"/>
+      <c r="E12" s="285" t="n"/>
+      <c r="F12" s="690" t="inlineStr">
         <is>
           <t>Record Status</t>
         </is>
       </c>
-      <c r="G12" s="22" t="n"/>
-      <c r="H12" s="658" t="inlineStr"/>
-      <c r="I12" s="19" t="n"/>
-      <c r="J12" s="22" t="n"/>
+      <c r="G12" s="285" t="n"/>
+      <c r="H12" s="694" t="inlineStr"/>
+      <c r="I12" s="283" t="n"/>
+      <c r="J12" s="285" t="n"/>
       <c r="K12" s="660" t="n"/>
       <c r="L12" s="660" t="n"/>
       <c r="M12" s="660" t="n"/>
@@ -7411,15 +7424,15 @@
           <t>2.  COMMERCIAL AND TECHNICAL SCREENING</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n"/>
-      <c r="C14" s="27" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="27" t="n"/>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="27" t="n"/>
-      <c r="H14" s="27" t="n"/>
-      <c r="I14" s="27" t="n"/>
-      <c r="J14" s="27" t="n"/>
+      <c r="B14" s="289" t="n"/>
+      <c r="C14" s="289" t="n"/>
+      <c r="D14" s="289" t="n"/>
+      <c r="E14" s="289" t="n"/>
+      <c r="F14" s="289" t="n"/>
+      <c r="G14" s="289" t="n"/>
+      <c r="H14" s="289" t="n"/>
+      <c r="I14" s="289" t="n"/>
+      <c r="J14" s="289" t="n"/>
       <c r="K14" s="643" t="n"/>
       <c r="L14" s="643" t="n"/>
       <c r="M14" s="643" t="n"/>
@@ -7452,24 +7465,24 @@
       <c r="AN14" s="644" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="645" t="inlineStr">
+      <c r="A15" s="685" t="inlineStr">
         <is>
           <t>Current Scope</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="646" t="inlineStr"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="647" t="inlineStr">
+      <c r="B15" s="272" t="n"/>
+      <c r="C15" s="331" t="inlineStr"/>
+      <c r="D15" s="271" t="n"/>
+      <c r="E15" s="272" t="n"/>
+      <c r="F15" s="686" t="inlineStr">
         <is>
           <t>Review Summary</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="646" t="inlineStr"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="6" t="n"/>
+      <c r="G15" s="272" t="n"/>
+      <c r="H15" s="331" t="inlineStr"/>
+      <c r="I15" s="271" t="n"/>
+      <c r="J15" s="272" t="n"/>
       <c r="K15" s="648" t="n"/>
       <c r="L15" s="648" t="n"/>
       <c r="M15" s="648" t="n"/>
@@ -7502,24 +7515,24 @@
       <c r="AN15" s="649" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="650" t="inlineStr">
+      <c r="A16" s="687" t="inlineStr">
         <is>
           <t>Top Risk / Constraint</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n"/>
-      <c r="C16" s="651" t="inlineStr"/>
-      <c r="D16" s="12" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="652" t="inlineStr">
+      <c r="B16" s="278" t="n"/>
+      <c r="C16" s="693" t="inlineStr"/>
+      <c r="D16" s="277" t="n"/>
+      <c r="E16" s="278" t="n"/>
+      <c r="F16" s="688" t="inlineStr">
         <is>
           <t>Next Review</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n"/>
-      <c r="H16" s="651" t="inlineStr"/>
-      <c r="I16" s="12" t="n"/>
-      <c r="J16" s="13" t="n"/>
+      <c r="G16" s="278" t="n"/>
+      <c r="H16" s="693" t="inlineStr"/>
+      <c r="I16" s="277" t="n"/>
+      <c r="J16" s="278" t="n"/>
       <c r="K16" s="653" t="n"/>
       <c r="L16" s="653" t="n"/>
       <c r="M16" s="653" t="n"/>
@@ -7552,24 +7565,24 @@
       <c r="AN16" s="654" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="650" t="inlineStr">
+      <c r="A17" s="687" t="inlineStr">
         <is>
           <t>Action Owner</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n"/>
-      <c r="C17" s="651" t="inlineStr"/>
-      <c r="D17" s="12" t="n"/>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="652" t="inlineStr">
+      <c r="B17" s="278" t="n"/>
+      <c r="C17" s="693" t="inlineStr"/>
+      <c r="D17" s="277" t="n"/>
+      <c r="E17" s="278" t="n"/>
+      <c r="F17" s="688" t="inlineStr">
         <is>
           <t>Next Review Date</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n"/>
-      <c r="H17" s="651" t="inlineStr"/>
-      <c r="I17" s="12" t="n"/>
-      <c r="J17" s="13" t="n"/>
+      <c r="G17" s="278" t="n"/>
+      <c r="H17" s="693" t="inlineStr"/>
+      <c r="I17" s="277" t="n"/>
+      <c r="J17" s="278" t="n"/>
       <c r="K17" s="653" t="n"/>
       <c r="L17" s="653" t="n"/>
       <c r="M17" s="653" t="n"/>
@@ -7602,24 +7615,24 @@
       <c r="AN17" s="654" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="657" t="inlineStr">
+      <c r="A18" s="689" t="inlineStr">
         <is>
           <t>Escalation if Overdue</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="658" t="inlineStr"/>
-      <c r="D18" s="19" t="n"/>
-      <c r="E18" s="22" t="n"/>
-      <c r="F18" s="659" t="inlineStr">
+      <c r="B18" s="285" t="n"/>
+      <c r="C18" s="694" t="inlineStr"/>
+      <c r="D18" s="283" t="n"/>
+      <c r="E18" s="285" t="n"/>
+      <c r="F18" s="690" t="inlineStr">
         <is>
           <t>Overall Status</t>
         </is>
       </c>
-      <c r="G18" s="22" t="n"/>
-      <c r="H18" s="658" t="inlineStr"/>
-      <c r="I18" s="19" t="n"/>
-      <c r="J18" s="22" t="n"/>
+      <c r="G18" s="285" t="n"/>
+      <c r="H18" s="694" t="inlineStr"/>
+      <c r="I18" s="283" t="n"/>
+      <c r="J18" s="285" t="n"/>
       <c r="K18" s="660" t="n"/>
       <c r="L18" s="660" t="n"/>
       <c r="M18" s="660" t="n"/>
@@ -7699,15 +7712,15 @@
           <t>3.  RISK AND RESPONSE SECTION</t>
         </is>
       </c>
-      <c r="B20" s="27" t="n"/>
-      <c r="C20" s="27" t="n"/>
-      <c r="D20" s="27" t="n"/>
-      <c r="E20" s="27" t="n"/>
-      <c r="F20" s="27" t="n"/>
-      <c r="G20" s="27" t="n"/>
-      <c r="H20" s="27" t="n"/>
-      <c r="I20" s="27" t="n"/>
-      <c r="J20" s="27" t="n"/>
+      <c r="B20" s="289" t="n"/>
+      <c r="C20" s="289" t="n"/>
+      <c r="D20" s="289" t="n"/>
+      <c r="E20" s="289" t="n"/>
+      <c r="F20" s="289" t="n"/>
+      <c r="G20" s="289" t="n"/>
+      <c r="H20" s="289" t="n"/>
+      <c r="I20" s="289" t="n"/>
+      <c r="J20" s="289" t="n"/>
       <c r="K20" s="643" t="n"/>
       <c r="L20" s="643" t="n"/>
       <c r="M20" s="643" t="n"/>
@@ -8679,15 +8692,15 @@
           <t>4.  QUOTE OUTCOME LOG</t>
         </is>
       </c>
-      <c r="B41" s="27" t="n"/>
-      <c r="C41" s="27" t="n"/>
-      <c r="D41" s="27" t="n"/>
-      <c r="E41" s="27" t="n"/>
-      <c r="F41" s="27" t="n"/>
-      <c r="G41" s="27" t="n"/>
-      <c r="H41" s="27" t="n"/>
-      <c r="I41" s="27" t="n"/>
-      <c r="J41" s="27" t="n"/>
+      <c r="B41" s="289" t="n"/>
+      <c r="C41" s="289" t="n"/>
+      <c r="D41" s="289" t="n"/>
+      <c r="E41" s="289" t="n"/>
+      <c r="F41" s="289" t="n"/>
+      <c r="G41" s="289" t="n"/>
+      <c r="H41" s="289" t="n"/>
+      <c r="I41" s="289" t="n"/>
+      <c r="J41" s="289" t="n"/>
       <c r="K41" s="643" t="n"/>
       <c r="L41" s="643" t="n"/>
       <c r="M41" s="643" t="n"/>
@@ -8720,28 +8733,28 @@
       <c r="AN41" s="644" t="n"/>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="674" t="inlineStr">
+      <c r="A42" s="695" t="inlineStr">
         <is>
           <t>Periodic review</t>
         </is>
       </c>
-      <c r="B42" s="5" t="n"/>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="675" t="inlineStr">
+      <c r="B42" s="271" t="n"/>
+      <c r="C42" s="272" t="n"/>
+      <c r="D42" s="696" t="inlineStr">
         <is>
           <t>Open items / escalation</t>
         </is>
       </c>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="675" t="inlineStr">
+      <c r="E42" s="271" t="n"/>
+      <c r="F42" s="272" t="n"/>
+      <c r="G42" s="696" t="inlineStr">
         <is>
           <t>Approval / archive</t>
         </is>
       </c>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="6" t="n"/>
+      <c r="H42" s="271" t="n"/>
+      <c r="I42" s="271" t="n"/>
+      <c r="J42" s="272" t="n"/>
       <c r="K42" s="648" t="n"/>
       <c r="L42" s="648" t="n"/>
       <c r="M42" s="648" t="n"/>
@@ -8774,30 +8787,26 @@
       <c r="AN42" s="649" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="213" t="inlineStr">
+      <c r="A43" s="697" t="inlineStr">
         <is>
           <t>Rolling RFQ intake and quote-outcome memory only; do not replace Epicor commercial master.
 Review owner: _____________________________________________</t>
         </is>
       </c>
-      <c r="B43" s="12" t="n"/>
-      <c r="C43" s="13" t="n"/>
-      <c r="D43" s="14" t="inlineStr">
+      <c r="C43" s="698" t="n"/>
+      <c r="D43" s="296" t="inlineStr">
         <is>
           <t>Final evidence ref: ________________________________________
 Outstanding items / actions: ________________________________</t>
         </is>
       </c>
-      <c r="E43" s="12" t="n"/>
-      <c r="F43" s="13" t="n"/>
-      <c r="G43" s="196" t="inlineStr">
+      <c r="F43" s="698" t="n"/>
+      <c r="G43" s="699" t="inlineStr">
         <is>
           <t>Name / Signature / Date</t>
         </is>
       </c>
-      <c r="H43" s="12" t="n"/>
-      <c r="I43" s="12" t="n"/>
-      <c r="J43" s="13" t="n"/>
+      <c r="J43" s="698" t="n"/>
       <c r="K43" s="653" t="n"/>
       <c r="L43" s="653" t="n"/>
       <c r="M43" s="653" t="n"/>
@@ -8830,16 +8839,10 @@
       <c r="AN43" s="654" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="16" t="n"/>
-      <c r="B44" s="12" t="n"/>
-      <c r="C44" s="13" t="n"/>
-      <c r="D44" s="12" t="n"/>
-      <c r="E44" s="12" t="n"/>
-      <c r="F44" s="13" t="n"/>
-      <c r="G44" s="12" t="n"/>
-      <c r="H44" s="12" t="n"/>
-      <c r="I44" s="12" t="n"/>
-      <c r="J44" s="13" t="n"/>
+      <c r="A44" s="275" t="n"/>
+      <c r="C44" s="698" t="n"/>
+      <c r="F44" s="698" t="n"/>
+      <c r="J44" s="698" t="n"/>
       <c r="K44" s="653" t="n"/>
       <c r="L44" s="653" t="n"/>
       <c r="M44" s="653" t="n"/>
@@ -8872,16 +8875,10 @@
       <c r="AN44" s="654" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="16" t="n"/>
-      <c r="B45" s="12" t="n"/>
-      <c r="C45" s="13" t="n"/>
-      <c r="D45" s="12" t="n"/>
-      <c r="E45" s="12" t="n"/>
-      <c r="F45" s="13" t="n"/>
-      <c r="G45" s="12" t="n"/>
-      <c r="H45" s="12" t="n"/>
-      <c r="I45" s="12" t="n"/>
-      <c r="J45" s="13" t="n"/>
+      <c r="A45" s="275" t="n"/>
+      <c r="C45" s="698" t="n"/>
+      <c r="F45" s="698" t="n"/>
+      <c r="J45" s="698" t="n"/>
       <c r="K45" s="653" t="n"/>
       <c r="L45" s="653" t="n"/>
       <c r="M45" s="653" t="n"/>
@@ -8914,16 +8911,16 @@
       <c r="AN45" s="654" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="18" t="n"/>
-      <c r="B46" s="19" t="n"/>
-      <c r="C46" s="22" t="n"/>
-      <c r="D46" s="19" t="n"/>
-      <c r="E46" s="19" t="n"/>
-      <c r="F46" s="22" t="n"/>
-      <c r="G46" s="19" t="n"/>
-      <c r="H46" s="19" t="n"/>
-      <c r="I46" s="19" t="n"/>
-      <c r="J46" s="22" t="n"/>
+      <c r="A46" s="281" t="n"/>
+      <c r="B46" s="277" t="n"/>
+      <c r="C46" s="278" t="n"/>
+      <c r="D46" s="277" t="n"/>
+      <c r="E46" s="277" t="n"/>
+      <c r="F46" s="278" t="n"/>
+      <c r="G46" s="277" t="n"/>
+      <c r="H46" s="277" t="n"/>
+      <c r="I46" s="277" t="n"/>
+      <c r="J46" s="278" t="n"/>
       <c r="K46" s="660" t="n"/>
       <c r="L46" s="660" t="n"/>
       <c r="M46" s="660" t="n"/>
@@ -8961,15 +8958,15 @@
           <t>NOTICE  —  Enter data only in designated white input cells. One form per event or job unless this workbook is designated as rolling. Do not add, delete or resize columns/rows. File naming: FRM-201_[RECORDID]_[YYYYMMDD].xlsx | Controlled source sets: Epicor / M365 / approved ANNEX references only.</t>
         </is>
       </c>
-      <c r="B47" s="27" t="n"/>
-      <c r="C47" s="27" t="n"/>
-      <c r="D47" s="27" t="n"/>
-      <c r="E47" s="27" t="n"/>
-      <c r="F47" s="27" t="n"/>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="27" t="n"/>
-      <c r="I47" s="27" t="n"/>
-      <c r="J47" s="27" t="n"/>
+      <c r="B47" s="289" t="n"/>
+      <c r="C47" s="289" t="n"/>
+      <c r="D47" s="289" t="n"/>
+      <c r="E47" s="289" t="n"/>
+      <c r="F47" s="289" t="n"/>
+      <c r="G47" s="289" t="n"/>
+      <c r="H47" s="289" t="n"/>
+      <c r="I47" s="289" t="n"/>
+      <c r="J47" s="289" t="n"/>
       <c r="K47" s="643" t="n"/>
       <c r="L47" s="643" t="n"/>
       <c r="M47" s="643" t="n"/>
@@ -9282,7 +9279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CU7"/>
+  <dimension ref="A1:AN7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>
@@ -9918,7 +9915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CU8"/>
+  <dimension ref="A1:AN8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>
@@ -10641,15 +10638,15 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="340" t="n"/>
-      <c r="B1" s="53" t="n"/>
+      <c r="A1" s="412" t="n"/>
+      <c r="B1" s="310" t="n"/>
       <c r="C1" s="3" t="inlineStr">
         <is>
           <t>FILTER VIEW / REVIEW CONFIGURATION</t>
         </is>
       </c>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
+      <c r="D1" s="268" t="n"/>
+      <c r="E1" s="268" t="n"/>
       <c r="F1" s="676" t="inlineStr">
         <is>
           <t>Form Code</t>
@@ -10695,11 +10692,9 @@
       <c r="AN1" s="625" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="9" t="n"/>
-      <c r="B2" s="54" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
+      <c r="A2" s="275" t="n"/>
+      <c r="B2" s="312" t="n"/>
+      <c r="C2" s="275" t="n"/>
       <c r="F2" s="679" t="inlineStr">
         <is>
           <t>Revision</t>
@@ -10745,11 +10740,9 @@
       <c r="AN2" s="630" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="54" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
+      <c r="A3" s="275" t="n"/>
+      <c r="B3" s="312" t="n"/>
+      <c r="C3" s="275" t="n"/>
       <c r="F3" s="679" t="inlineStr">
         <is>
           <t>Eff. Date</t>
@@ -10795,15 +10788,13 @@
       <c r="AN3" s="630" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="9" t="n"/>
-      <c r="B4" s="54" t="n"/>
+      <c r="A4" s="275" t="n"/>
+      <c r="B4" s="312" t="n"/>
       <c r="C4" s="631" t="inlineStr">
         <is>
           <t>Quality Management System  ·  Controlled Document</t>
         </is>
       </c>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
       <c r="F4" s="679" t="inlineStr">
         <is>
           <t>Owner</t>
@@ -10849,15 +10840,15 @@
       <c r="AN4" s="630" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="18" t="n"/>
-      <c r="B5" s="24" t="n"/>
+      <c r="A5" s="282" t="n"/>
+      <c r="B5" s="287" t="n"/>
       <c r="C5" s="634" t="inlineStr">
         <is>
           <t>HESEM Engineering  ·  ISO 9001 / AS9100  ·  Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="19" t="n"/>
+      <c r="D5" s="283" t="n"/>
+      <c r="E5" s="283" t="n"/>
       <c r="F5" s="682" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -10950,12 +10941,12 @@
           <t>1.  CONTROL CONTEXT / SUPPORT TAB PURPOSE</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n"/>
-      <c r="C7" s="27" t="n"/>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
+      <c r="B7" s="289" t="n"/>
+      <c r="C7" s="289" t="n"/>
+      <c r="D7" s="289" t="n"/>
+      <c r="E7" s="289" t="n"/>
+      <c r="F7" s="289" t="n"/>
+      <c r="G7" s="289" t="n"/>
       <c r="H7" s="643" t="n"/>
       <c r="I7" s="643" t="n"/>
       <c r="J7" s="643" t="n"/>
@@ -10996,24 +10987,24 @@
           <t>Parent Form</t>
         </is>
       </c>
-      <c r="B8" s="646" t="inlineStr">
+      <c r="B8" s="331" t="inlineStr">
         <is>
           <t>FRM-201 · RFQ REGISTER</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="6" t="n"/>
+      <c r="C8" s="271" t="n"/>
+      <c r="D8" s="272" t="n"/>
       <c r="E8" s="686" t="inlineStr">
         <is>
           <t>Support Tab</t>
         </is>
       </c>
-      <c r="F8" s="646" t="inlineStr">
+      <c r="F8" s="331" t="inlineStr">
         <is>
           <t>FILTER_VIEW</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n"/>
+      <c r="G8" s="272" t="n"/>
       <c r="H8" s="648" t="n"/>
       <c r="I8" s="648" t="n"/>
       <c r="J8" s="648" t="n"/>
@@ -11054,24 +11045,24 @@
           <t>Tab Purpose</t>
         </is>
       </c>
-      <c r="B9" s="651" t="inlineStr">
+      <c r="B9" s="693" t="inlineStr">
         <is>
           <t>Controlled saved-filter and review-view guidance for rolling review. Do not use as a transaction replacement.</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="13" t="n"/>
+      <c r="C9" s="277" t="n"/>
+      <c r="D9" s="278" t="n"/>
       <c r="E9" s="688" t="inlineStr">
         <is>
           <t>Working Owner</t>
         </is>
       </c>
-      <c r="F9" s="651" t="inlineStr">
+      <c r="F9" s="693" t="inlineStr">
         <is>
           <t>Sales / Commercial</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n"/>
+      <c r="G9" s="278" t="n"/>
       <c r="H9" s="653" t="n"/>
       <c r="I9" s="653" t="n"/>
       <c r="J9" s="653" t="n"/>
@@ -11112,24 +11103,24 @@
           <t>Source of Truth</t>
         </is>
       </c>
-      <c r="B10" s="651" t="inlineStr">
+      <c r="B10" s="693" t="inlineStr">
         <is>
           <t>Use controlled parent-form references, _IMPORT lists and approved evidence sources only.</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="13" t="n"/>
+      <c r="C10" s="277" t="n"/>
+      <c r="D10" s="278" t="n"/>
       <c r="E10" s="688" t="inlineStr">
         <is>
           <t>Reviewed By</t>
         </is>
       </c>
-      <c r="F10" s="651" t="inlineStr">
+      <c r="F10" s="693" t="inlineStr">
         <is>
           <t>Commercial Manager</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n"/>
+      <c r="G10" s="278" t="n"/>
       <c r="H10" s="653" t="n"/>
       <c r="I10" s="653" t="n"/>
       <c r="J10" s="653" t="n"/>
@@ -11170,24 +11161,24 @@
           <t>Update Trigger</t>
         </is>
       </c>
-      <c r="B11" s="651" t="inlineStr">
+      <c r="B11" s="693" t="inlineStr">
         <is>
           <t>Update when the linked review, evidence or follow-up status changes.</t>
         </is>
       </c>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="13" t="n"/>
+      <c r="C11" s="277" t="n"/>
+      <c r="D11" s="278" t="n"/>
       <c r="E11" s="688" t="inlineStr">
         <is>
           <t>Data Structure</t>
         </is>
       </c>
-      <c r="F11" s="651" t="inlineStr">
+      <c r="F11" s="693" t="inlineStr">
         <is>
           <t>Structured Excel Table with filters and print-title rows.</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n"/>
+      <c r="G11" s="278" t="n"/>
       <c r="H11" s="655" t="n"/>
       <c r="I11" s="655" t="n"/>
       <c r="J11" s="655" t="n"/>
@@ -11228,24 +11219,24 @@
           <t>Retention Rule</t>
         </is>
       </c>
-      <c r="B12" s="658" t="inlineStr">
+      <c r="B12" s="694" t="inlineStr">
         <is>
           <t>Do not delete historical lines once evidence has been recorded or reviewed.</t>
         </is>
       </c>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="22" t="n"/>
+      <c r="C12" s="283" t="n"/>
+      <c r="D12" s="285" t="n"/>
       <c r="E12" s="690" t="inlineStr">
         <is>
           <t>Controlled Status</t>
         </is>
       </c>
-      <c r="F12" s="658" t="inlineStr">
+      <c r="F12" s="694" t="inlineStr">
         <is>
           <t>Support sheet only — not a replacement for ERP / M365 system-of-record.</t>
         </is>
       </c>
-      <c r="G12" s="22" t="n"/>
+      <c r="G12" s="285" t="n"/>
       <c r="H12" s="660" t="n"/>
       <c r="I12" s="660" t="n"/>
       <c r="J12" s="660" t="n"/>
@@ -11328,12 +11319,12 @@
           <t>2.  WORKING TABLE / DETAIL LINES</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n"/>
-      <c r="C14" s="27" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="27" t="n"/>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="27" t="n"/>
+      <c r="B14" s="289" t="n"/>
+      <c r="C14" s="289" t="n"/>
+      <c r="D14" s="289" t="n"/>
+      <c r="E14" s="289" t="n"/>
+      <c r="F14" s="289" t="n"/>
+      <c r="G14" s="289" t="n"/>
       <c r="H14" s="643" t="n"/>
       <c r="I14" s="643" t="n"/>
       <c r="J14" s="643" t="n"/>
@@ -11374,12 +11365,12 @@
           <t>Controlled saved-filter and review-view guidance for rolling review. Do not use as a transaction replacement.</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n"/>
-      <c r="C15" s="27" t="n"/>
-      <c r="D15" s="27" t="n"/>
-      <c r="E15" s="27" t="n"/>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="27" t="n"/>
+      <c r="B15" s="289" t="n"/>
+      <c r="C15" s="289" t="n"/>
+      <c r="D15" s="289" t="n"/>
+      <c r="E15" s="289" t="n"/>
+      <c r="F15" s="289" t="n"/>
+      <c r="G15" s="289" t="n"/>
       <c r="H15" s="643" t="n"/>
       <c r="I15" s="643" t="n"/>
       <c r="J15" s="643" t="n"/>
@@ -11892,12 +11883,12 @@
           <t>NOTICE  —  Controlled saved-filter and review-view guidance for rolling review. Do not use as a transaction replacement.  Maintain traceability to the parent form and approved evidence references. Do not add, delete or resize structured columns. Keep dropdown values, review dates and status fields controlled.</t>
         </is>
       </c>
-      <c r="B26" s="27" t="n"/>
-      <c r="C26" s="27" t="n"/>
-      <c r="D26" s="27" t="n"/>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="27" t="n"/>
-      <c r="G26" s="27" t="n"/>
+      <c r="B26" s="289" t="n"/>
+      <c r="C26" s="289" t="n"/>
+      <c r="D26" s="289" t="n"/>
+      <c r="E26" s="289" t="n"/>
+      <c r="F26" s="289" t="n"/>
+      <c r="G26" s="289" t="n"/>
       <c r="H26" s="643" t="n"/>
       <c r="I26" s="643" t="n"/>
       <c r="J26" s="643" t="n"/>
@@ -12218,16 +12209,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1">
-      <c r="A1" s="340" t="n"/>
-      <c r="B1" s="53" t="n"/>
+      <c r="A1" s="412" t="n"/>
+      <c r="B1" s="310" t="n"/>
       <c r="C1" s="3" t="inlineStr">
         <is>
           <t>PERIODIC REVIEW RECORD</t>
         </is>
       </c>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
+      <c r="D1" s="268" t="n"/>
+      <c r="E1" s="268" t="n"/>
+      <c r="F1" s="268" t="n"/>
       <c r="G1" s="676" t="inlineStr">
         <is>
           <t>Form Code</t>
@@ -12272,12 +12263,9 @@
       <c r="AN1" s="625" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="9" t="n"/>
-      <c r="B2" s="54" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
+      <c r="A2" s="275" t="n"/>
+      <c r="B2" s="312" t="n"/>
+      <c r="C2" s="275" t="n"/>
       <c r="G2" s="679" t="inlineStr">
         <is>
           <t>Revision</t>
@@ -12322,12 +12310,9 @@
       <c r="AN2" s="630" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="54" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
+      <c r="A3" s="275" t="n"/>
+      <c r="B3" s="312" t="n"/>
+      <c r="C3" s="275" t="n"/>
       <c r="G3" s="679" t="inlineStr">
         <is>
           <t>Eff. Date</t>
@@ -12372,16 +12357,13 @@
       <c r="AN3" s="630" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="9" t="n"/>
-      <c r="B4" s="54" t="n"/>
+      <c r="A4" s="275" t="n"/>
+      <c r="B4" s="312" t="n"/>
       <c r="C4" s="631" t="inlineStr">
         <is>
           <t>Quality Management System  ·  Controlled Document</t>
         </is>
       </c>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
       <c r="G4" s="679" t="inlineStr">
         <is>
           <t>Owner</t>
@@ -12426,16 +12408,16 @@
       <c r="AN4" s="630" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="18" t="n"/>
-      <c r="B5" s="24" t="n"/>
+      <c r="A5" s="282" t="n"/>
+      <c r="B5" s="287" t="n"/>
       <c r="C5" s="634" t="inlineStr">
         <is>
           <t>HESEM Engineering  ·  ISO 9001 / AS9100  ·  Semiconductor Equipment Parts</t>
         </is>
       </c>
-      <c r="D5" s="19" t="n"/>
-      <c r="E5" s="19" t="n"/>
-      <c r="F5" s="19" t="n"/>
+      <c r="D5" s="283" t="n"/>
+      <c r="E5" s="283" t="n"/>
+      <c r="F5" s="283" t="n"/>
       <c r="G5" s="682" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -12527,13 +12509,13 @@
           <t>1.  CONTROL CONTEXT / SUPPORT TAB PURPOSE</t>
         </is>
       </c>
-      <c r="B7" s="27" t="n"/>
-      <c r="C7" s="27" t="n"/>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
-      <c r="H7" s="27" t="n"/>
+      <c r="B7" s="289" t="n"/>
+      <c r="C7" s="289" t="n"/>
+      <c r="D7" s="289" t="n"/>
+      <c r="E7" s="289" t="n"/>
+      <c r="F7" s="289" t="n"/>
+      <c r="G7" s="289" t="n"/>
+      <c r="H7" s="289" t="n"/>
       <c r="I7" s="643" t="n"/>
       <c r="J7" s="643" t="n"/>
       <c r="K7" s="643" t="n"/>
@@ -12568,30 +12550,30 @@
       <c r="AN7" s="644" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="645" t="inlineStr">
+      <c r="A8" s="685" t="inlineStr">
         <is>
           <t>Parent Form</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n"/>
-      <c r="C8" s="646" t="inlineStr">
+      <c r="B8" s="272" t="n"/>
+      <c r="C8" s="331" t="inlineStr">
         <is>
           <t>FRM-201 · RFQ REGISTER</t>
         </is>
       </c>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="647" t="inlineStr">
+      <c r="D8" s="272" t="n"/>
+      <c r="E8" s="686" t="inlineStr">
         <is>
           <t>Support Tab</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="646" t="inlineStr">
+      <c r="F8" s="272" t="n"/>
+      <c r="G8" s="331" t="inlineStr">
         <is>
           <t>PERIOD_REVIEW</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n"/>
+      <c r="H8" s="272" t="n"/>
       <c r="I8" s="648" t="n"/>
       <c r="J8" s="648" t="n"/>
       <c r="K8" s="648" t="n"/>
@@ -12626,30 +12608,30 @@
       <c r="AN8" s="649" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="650" t="inlineStr">
+      <c r="A9" s="687" t="inlineStr">
         <is>
           <t>Tab Purpose</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n"/>
-      <c r="C9" s="651" t="inlineStr">
+      <c r="B9" s="278" t="n"/>
+      <c r="C9" s="693" t="inlineStr">
         <is>
           <t>Formal periodic review and cadence record for the rolling workbook.</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="652" t="inlineStr">
+      <c r="D9" s="278" t="n"/>
+      <c r="E9" s="688" t="inlineStr">
         <is>
           <t>Working Owner</t>
         </is>
       </c>
-      <c r="F9" s="13" t="n"/>
-      <c r="G9" s="651" t="inlineStr">
+      <c r="F9" s="278" t="n"/>
+      <c r="G9" s="693" t="inlineStr">
         <is>
           <t>Sales / Commercial</t>
         </is>
       </c>
-      <c r="H9" s="13" t="n"/>
+      <c r="H9" s="278" t="n"/>
       <c r="I9" s="653" t="n"/>
       <c r="J9" s="653" t="n"/>
       <c r="K9" s="653" t="n"/>
@@ -12684,30 +12666,30 @@
       <c r="AN9" s="654" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="650" t="inlineStr">
+      <c r="A10" s="687" t="inlineStr">
         <is>
           <t>Source of Truth</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n"/>
-      <c r="C10" s="651" t="inlineStr">
+      <c r="B10" s="278" t="n"/>
+      <c r="C10" s="693" t="inlineStr">
         <is>
           <t>Use controlled parent-form references, _IMPORT lists and approved evidence sources only.</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="652" t="inlineStr">
+      <c r="D10" s="278" t="n"/>
+      <c r="E10" s="688" t="inlineStr">
         <is>
           <t>Reviewed By</t>
         </is>
       </c>
-      <c r="F10" s="13" t="n"/>
-      <c r="G10" s="651" t="inlineStr">
+      <c r="F10" s="278" t="n"/>
+      <c r="G10" s="693" t="inlineStr">
         <is>
           <t>Commercial Manager</t>
         </is>
       </c>
-      <c r="H10" s="13" t="n"/>
+      <c r="H10" s="278" t="n"/>
       <c r="I10" s="653" t="n"/>
       <c r="J10" s="653" t="n"/>
       <c r="K10" s="653" t="n"/>
@@ -12742,30 +12724,30 @@
       <c r="AN10" s="654" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="650" t="inlineStr">
+      <c r="A11" s="687" t="inlineStr">
         <is>
           <t>Update Trigger</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="651" t="inlineStr">
+      <c r="B11" s="278" t="n"/>
+      <c r="C11" s="693" t="inlineStr">
         <is>
           <t>Update when the linked review, evidence or follow-up status changes.</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="652" t="inlineStr">
+      <c r="D11" s="278" t="n"/>
+      <c r="E11" s="688" t="inlineStr">
         <is>
           <t>Data Structure</t>
         </is>
       </c>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="651" t="inlineStr">
+      <c r="F11" s="278" t="n"/>
+      <c r="G11" s="693" t="inlineStr">
         <is>
           <t>Structured Excel Table with filters and print-title rows.</t>
         </is>
       </c>
-      <c r="H11" s="13" t="n"/>
+      <c r="H11" s="278" t="n"/>
       <c r="I11" s="655" t="n"/>
       <c r="J11" s="655" t="n"/>
       <c r="K11" s="655" t="n"/>
@@ -12800,30 +12782,30 @@
       <c r="AN11" s="656" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="657" t="inlineStr">
+      <c r="A12" s="689" t="inlineStr">
         <is>
           <t>Retention Rule</t>
         </is>
       </c>
-      <c r="B12" s="22" t="n"/>
-      <c r="C12" s="658" t="inlineStr">
+      <c r="B12" s="285" t="n"/>
+      <c r="C12" s="694" t="inlineStr">
         <is>
           <t>Do not delete historical lines once evidence has been recorded or reviewed.</t>
         </is>
       </c>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="659" t="inlineStr">
+      <c r="D12" s="285" t="n"/>
+      <c r="E12" s="690" t="inlineStr">
         <is>
           <t>Controlled Status</t>
         </is>
       </c>
-      <c r="F12" s="22" t="n"/>
-      <c r="G12" s="658" t="inlineStr">
+      <c r="F12" s="285" t="n"/>
+      <c r="G12" s="694" t="inlineStr">
         <is>
           <t>Support sheet only — not a replacement for ERP / M365 system-of-record.</t>
         </is>
       </c>
-      <c r="H12" s="22" t="n"/>
+      <c r="H12" s="285" t="n"/>
       <c r="I12" s="660" t="n"/>
       <c r="J12" s="660" t="n"/>
       <c r="K12" s="660" t="n"/>
@@ -12905,13 +12887,13 @@
           <t>2.  WORKING TABLE / DETAIL LINES</t>
         </is>
       </c>
-      <c r="B14" s="27" t="n"/>
-      <c r="C14" s="27" t="n"/>
-      <c r="D14" s="27" t="n"/>
-      <c r="E14" s="27" t="n"/>
-      <c r="F14" s="27" t="n"/>
-      <c r="G14" s="27" t="n"/>
-      <c r="H14" s="27" t="n"/>
+      <c r="B14" s="289" t="n"/>
+      <c r="C14" s="289" t="n"/>
+      <c r="D14" s="289" t="n"/>
+      <c r="E14" s="289" t="n"/>
+      <c r="F14" s="289" t="n"/>
+      <c r="G14" s="289" t="n"/>
+      <c r="H14" s="289" t="n"/>
       <c r="I14" s="643" t="n"/>
       <c r="J14" s="643" t="n"/>
       <c r="K14" s="643" t="n"/>
@@ -12951,13 +12933,13 @@
           <t>Formal periodic review and cadence record for the rolling workbook.</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n"/>
-      <c r="C15" s="27" t="n"/>
-      <c r="D15" s="27" t="n"/>
-      <c r="E15" s="27" t="n"/>
-      <c r="F15" s="27" t="n"/>
-      <c r="G15" s="27" t="n"/>
-      <c r="H15" s="27" t="n"/>
+      <c r="B15" s="289" t="n"/>
+      <c r="C15" s="289" t="n"/>
+      <c r="D15" s="289" t="n"/>
+      <c r="E15" s="289" t="n"/>
+      <c r="F15" s="289" t="n"/>
+      <c r="G15" s="289" t="n"/>
+      <c r="H15" s="289" t="n"/>
       <c r="I15" s="643" t="n"/>
       <c r="J15" s="643" t="n"/>
       <c r="K15" s="643" t="n"/>
@@ -13473,13 +13455,13 @@
           <t>NOTICE  —  Formal periodic review and cadence record for the rolling workbook.  Maintain traceability to the parent form and approved evidence references. Do not add, delete or resize structured columns. Keep dropdown values, review dates and status fields controlled.</t>
         </is>
       </c>
-      <c r="B26" s="27" t="n"/>
-      <c r="C26" s="27" t="n"/>
-      <c r="D26" s="27" t="n"/>
-      <c r="E26" s="27" t="n"/>
-      <c r="F26" s="27" t="n"/>
-      <c r="G26" s="27" t="n"/>
-      <c r="H26" s="27" t="n"/>
+      <c r="B26" s="289" t="n"/>
+      <c r="C26" s="289" t="n"/>
+      <c r="D26" s="289" t="n"/>
+      <c r="E26" s="289" t="n"/>
+      <c r="F26" s="289" t="n"/>
+      <c r="G26" s="289" t="n"/>
+      <c r="H26" s="289" t="n"/>
       <c r="I26" s="643" t="n"/>
       <c r="J26" s="643" t="n"/>
       <c r="K26" s="643" t="n"/>
@@ -13753,7 +13735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CU11"/>
+  <dimension ref="A1:AN11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.33" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
Remove freeze panes, sheet protection, and consolidate tabs for FRM-201
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/02-FRM-200/FRM-201_RFQ_Register.xlsx
+++ b/04-Bieu-Mau/02-FRM-200/FRM-201_RFQ_Register.xlsx
@@ -4,11 +4,11 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FRM-201_LOG" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_LISTS" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_IMPORT" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILTER_VIEW" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERIOD_REVIEW" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REF_LINKS" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_LISTS" sheetId="2" state="veryHidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_IMPORT" sheetId="3" state="veryHidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILTER_VIEW" sheetId="4" state="veryHidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERIOD_REVIEW" sheetId="5" state="veryHidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REF_LINKS" sheetId="6" state="veryHidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="VAL_STATUS_CORE">'_LISTS'!$A$2:$A$7</definedName>
@@ -7538,7 +7538,6 @@
       <c r="F24" s="388" t="n"/>
       <c r="G24" s="389" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="421" t="inlineStr">
         <is>
@@ -8246,7 +8245,6 @@
       <c r="G24" s="388" t="n"/>
       <c r="H24" s="389" t="n"/>
     </row>
-    <row r="25"/>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="421" t="inlineStr">
         <is>

</xml_diff>